<commit_message>
RESHIPPED (task261): the book asks re-cut on silent devices, the call held
cracker.py, run on the strict battery, kept all nine Ask A figures and
Ask B's three household counts: the PDS reversion, the partner
nominations and the merges are documented handling a careful solver
executes. Ask A is now held by a member's totals printed on each of
the member's pension rows (36 members, 12 in every group, beside 21
whose rows genuinely differ) and by six partners whose 2026 death the
annuity listing records but the client register does not. Ask B's
households are held by former partners still named on six
reversionary annuities. The cracker keeps 0 of 15, pair ceiling 37.0.

Five segments unchanged. checks 253, verify (43 figures), two builds
byte-identical, figures_check 198 of 198, precut 50 of 50. Judge pass
3 DETERMINISTIC, APPROVE; reader clean.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0142Jt4Mt622iBfGoK24ivCU
</commit_message>
<xml_diff>
--- a/task261/golden/retirement_segments_2027.xlsx
+++ b/task261/golden/retirement_segments_2027.xlsx
@@ -145,7 +145,7 @@
     <t>Each difference's standard error is taken from the difference itself, recomputed on every replicate weight and implicate. Committee's rule: neighbouring groups are kept apart where the difference is more than 1.96 times its standard error.</t>
   </si>
   <si>
-    <t>Our book: client register and annuity listing pulled 12 January 2027; pension extract and nominations at 31 December 2026. A pension whose member died before 31 December with a reversionary nominated is counted with the survivor; annuity income is the annual rate at 31 December 2026, deferred annuities not yet paying left out.</t>
+    <t>Our book: client register and annuity listing pulled 12 January 2027; pension extract and nominations at 31 December 2026. A pension whose member died before 31 December with a reversionary nominated is counted with the survivor; a partner whose 2026 death the annuity listing records is not counted, though the register still holds them; a member's pensions that repeat one balance and payment count once; annuity income is the annual rate at 31 December 2026, deferred annuities not yet paying left out.</t>
   </si>
   <si>
     <t>Dollar figures rounded to the nearest thousand.</t>
@@ -920,19 +920,19 @@
         <v>10</v>
       </c>
       <c r="B2">
-        <v>442</v>
+        <v>445</v>
       </c>
       <c r="C2" s="4">
-        <v>207655000</v>
+        <v>210509000</v>
       </c>
       <c r="D2" s="4">
-        <v>11448000</v>
+        <v>11589000</v>
       </c>
       <c r="E2">
-        <v>176</v>
+        <v>179</v>
       </c>
       <c r="F2" s="4">
-        <v>3606000</v>
+        <v>3653000</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
@@ -940,19 +940,19 @@
         <v>17</v>
       </c>
       <c r="B3" s="4">
-        <v>1168</v>
+        <v>1169</v>
       </c>
       <c r="C3" s="4">
-        <v>520479000</v>
+        <v>521126000</v>
       </c>
       <c r="D3" s="4">
-        <v>30320000</v>
+        <v>30350000</v>
       </c>
       <c r="E3">
-        <v>467</v>
+        <v>468</v>
       </c>
       <c r="F3" s="4">
-        <v>9011000</v>
+        <v>9041000</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
@@ -960,19 +960,19 @@
         <v>18</v>
       </c>
       <c r="B4">
-        <v>746</v>
+        <v>742</v>
       </c>
       <c r="C4" s="4">
-        <v>249568000</v>
+        <v>249685000</v>
       </c>
       <c r="D4" s="4">
-        <v>17994000</v>
+        <v>18003000</v>
       </c>
       <c r="E4">
-        <v>284</v>
+        <v>280</v>
       </c>
       <c r="F4" s="4">
-        <v>5614000</v>
+        <v>5510000</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
@@ -983,16 +983,16 @@
         <v>2356</v>
       </c>
       <c r="C5" s="6">
-        <v>977702000</v>
+        <v>981320000</v>
       </c>
       <c r="D5" s="6">
-        <v>59762000</v>
+        <v>59942000</v>
       </c>
       <c r="E5" s="2">
         <v>927</v>
       </c>
       <c r="F5" s="6">
-        <v>18231000</v>
+        <v>18204000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>